<commit_message>
Corrige les décalages de date UTC, refond le Gantt des missions et ajoute le champ modalité
- Corrige un décalage de date d'un jour (dashboard, jours fériés mobiles, fallbacks
  "aujourd'hui") causé par des allers-retours locaux -> UTC via toISOString()
- Refond l'onglet Missions admin : supprime la liste redondante, agrandit le Gantt
  avec repères hebdomadaires, ajoute un bouton de suppression dans la popup d'édition
- Ajoute le champ présentiel/distanciel au planning (UI + import/export Excel)
- Permet à l'admin de sélectionner une plage de jours sur la fiche alternant
  (comme côté alternant) et déplace l'import Excel dans "Modifier la fiche"
- Rend la surbrillance de sélection de plage visuellement distincte des couleurs
  de type de planning (bleu marine sombre au lieu d'une teinte proche de "Entreprise")

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/files/modele-planning.xlsx
+++ b/public/files/modele-planning.xlsx
@@ -398,11 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -411,6 +407,9 @@
       <c r="B1" t="str">
         <v>Type</v>
       </c>
+      <c r="C1" t="str">
+        <v>Modalité (si Entreprise)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -419,13 +418,19 @@
       <c r="B2" t="str">
         <v>entreprise</v>
       </c>
+      <c r="C2" t="str">
+        <v>presentiel</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
         <v>02/09/2025</v>
       </c>
       <c r="B3" t="str">
-        <v>ecole</v>
+        <v>entreprise</v>
+      </c>
+      <c r="C3" t="str">
+        <v>distanciel</v>
       </c>
     </row>
     <row r="4">
@@ -435,21 +440,20 @@
       <c r="B4" t="str">
         <v>ecole</v>
       </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
-  <cols>
-    <col min="1" max="1" width="40.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:B17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -485,40 +489,77 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>recuperation</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Jour de récupération</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v>absent</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B6" t="str">
         <v>Jour d'absence</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Remarques :</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>- Une ligne par jour.</v>
+        <v>Valeur à écrire dans la colonne Modalité</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Signification</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>- Le format de date doit être JJ/MM/AAAA.</v>
+        <v>presentiel</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Travail en présentiel (uniquement pour Entreprise)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>distanciel</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Travail en distanciel / télétravail (uniquement pour Entreprise)</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Remarques :</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>- Une ligne par jour.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>- Le format de date doit être JJ/MM/AAAA.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>- Ne modifiez pas les en-têtes de colonnes.</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="str">
+    <row r="16">
+      <c r="A16" t="str">
+        <v>- La colonne Modalité ne concerne que les jours de type Entreprise ; laissez-la vide sinon.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>- Supprimez les lignes d'exemple avant de remplir votre propre planning.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>